<commit_message>
feat(annoncetekster): auto-size column widths to fit content
fill-sheet.py now resizes every text column to its widest cell (capped at 60)
after writing copy, with LEN columns pinned at width 6. build-template.py
applies the same narrow/wide default to an empty template and drops the
hardcoded Campaign pre-seed (each run sets it from intake).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/inbound-cph/skills/annoncetekster/template.xlsx
+++ b/plugins/inbound-cph/skills/annoncetekster/template.xlsx
@@ -443,47 +443,47 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="6" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="6" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="6" customWidth="1" min="22" max="22"/>
     <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="6" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="6" customWidth="1" min="26" max="26"/>
     <col width="18" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="6" customWidth="1" min="28" max="28"/>
     <col width="18" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="6" customWidth="1" min="30" max="30"/>
     <col width="18" customWidth="1" min="31" max="31"/>
-    <col width="18" customWidth="1" min="32" max="32"/>
+    <col width="6" customWidth="1" min="32" max="32"/>
     <col width="18" customWidth="1" min="33" max="33"/>
-    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="6" customWidth="1" min="34" max="34"/>
     <col width="18" customWidth="1" min="35" max="35"/>
-    <col width="18" customWidth="1" min="36" max="36"/>
+    <col width="6" customWidth="1" min="36" max="36"/>
     <col width="18" customWidth="1" min="37" max="37"/>
-    <col width="18" customWidth="1" min="38" max="38"/>
+    <col width="6" customWidth="1" min="38" max="38"/>
     <col width="18" customWidth="1" min="39" max="39"/>
-    <col width="18" customWidth="1" min="40" max="40"/>
+    <col width="6" customWidth="1" min="40" max="40"/>
     <col width="18" customWidth="1" min="41" max="41"/>
-    <col width="18" customWidth="1" min="42" max="42"/>
+    <col width="6" customWidth="1" min="42" max="42"/>
     <col width="18" customWidth="1" min="43" max="43"/>
-    <col width="18" customWidth="1" min="44" max="44"/>
+    <col width="6" customWidth="1" min="44" max="44"/>
     <col width="18" customWidth="1" min="45" max="45"/>
-    <col width="18" customWidth="1" min="46" max="46"/>
+    <col width="6" customWidth="1" min="46" max="46"/>
     <col width="18" customWidth="1" min="47" max="47"/>
     <col width="18" customWidth="1" min="48" max="48"/>
   </cols>
@@ -731,11 +731,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>IC | GSN | Generic |</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>Responsive search ad</t>

</xml_diff>